<commit_message>
docs(perturbation): Mise à jour du planning + burnup global
</commit_message>
<xml_diff>
--- a/docs/artefact/J1/equipe-02-release-planning-v1.0.xlsx
+++ b/docs/artefact/J1/equipe-02-release-planning-v1.0.xlsx
@@ -1187,48 +1187,60 @@
       <c r="B5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>10</v>
+      <c r="C5" t="inlineStr" s="11">
+        <is>
+          <t>2</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>12</v>
+      <c r="C6" t="inlineStr" s="11">
+        <is>
+          <t>Adja Fatou SAGNA, Ousmane NDIAYE, Houda OUADAH, Danielle Jamila KOAGNE NGANKAM, Wicramachine SERGIO, Krishmini KULAKRISHNA, Mohammed DERKAOUI</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>14</v>
+      <c r="C7" t="inlineStr" s="11">
+        <is>
+          <t>cadrage</t>
+        </is>
       </c>
     </row>
     <row r="8" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>16</v>
+      <c r="C8" t="inlineStr" s="11">
+        <is>
+          <t>v1.0</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>18</v>
+      <c r="C9" t="inlineStr" s="11">
+        <is>
+          <t>29/06/2026 16h00</t>
+        </is>
       </c>
     </row>
     <row r="10" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>20</v>
+      <c r="C10" t="inlineStr" s="11">
+        <is>
+          <t>Validé PO</t>
+        </is>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">

</xml_diff>